<commit_message>
Update Master Journal workbook
</commit_message>
<xml_diff>
--- a/journal/Master Journal.xlsx
+++ b/journal/Master Journal.xlsx
@@ -23,11 +23,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.000&quot;R&quot;"/>
     <numFmt numFmtId="165" formatCode="#,##0.##########"/>
     <numFmt numFmtId="166" formatCode="#,##0.00 &quot;UNKNOWN&quot;"/>
     <numFmt numFmtId="167" formatCode="#,##0.00 &quot;AUD&quot;"/>
+    <numFmt numFmtId="168" formatCode="#,##0.########## &quot;USDT&quot;"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -293,7 +294,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -340,6 +341,7 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -727,7 +729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1531,6 +1533,21 @@
       <c r="D24" s="20" t="inlineStr">
         <is>
           <t>As Of</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Bybit Demo</t>
+        </is>
+      </c>
+      <c r="B25" s="46" t="n">
+        <v>371.30701792</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>USDT</t>
         </is>
       </c>
     </row>
@@ -1725,7 +1742,7 @@
       </c>
       <c r="I2" s="12" t="n"/>
       <c r="J2" s="12" t="n"/>
-      <c r="K2" s="34" t="n"/>
+      <c r="K2" s="35" t="n"/>
       <c r="L2" s="35" t="n">
         <v>-12.68</v>
       </c>
@@ -1803,7 +1820,7 @@
       </c>
       <c r="I3" s="17" t="n"/>
       <c r="J3" s="17" t="n"/>
-      <c r="K3" s="41" t="n"/>
+      <c r="K3" s="42" t="n"/>
       <c r="L3" s="42" t="n">
         <v>9.07</v>
       </c>

</xml_diff>